<commit_message>
add fig s14 and adapt tab s4
</commit_message>
<xml_diff>
--- a/data/random_collections/TabS4_readcount_breakdown.xlsx
+++ b/data/random_collections/TabS4_readcount_breakdown.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\briem\AppData\Roaming\MobaXterm\slash\RemoteFiles\591364_3_45\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\briem\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -16,6 +16,7 @@
     <sheet name="reads_per_library" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -3490,12 +3491,6 @@
     <t>alt_KOLF_old_TGCTGAGATCGG_r2.fq.gz</t>
   </si>
   <si>
-    <t>alt_KOLF_PTO_AACAGCGCCATG_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_AACAGCGCCATG_r2.fq.gz</t>
-  </si>
-  <si>
     <t>alt_KOLF_PTO_AAGCCTCAGTCC_r1.fq.gz</t>
   </si>
   <si>
@@ -3508,12 +3503,6 @@
     <t>alt_KOLF_PTO_AGTACCTTACGA_r2.fq.gz</t>
   </si>
   <si>
-    <t>alt_KOLF_PTO_AGTAGTTAGCCG_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_AGTAGTTAGCCG_r2.fq.gz</t>
-  </si>
-  <si>
     <t>alt_KOLF_PTO_CACCAAGACTTC_r1.fq.gz</t>
   </si>
   <si>
@@ -3526,30 +3515,12 @@
     <t>alt_KOLF_PTO_CGACCATACCTG_r2.fq.gz</t>
   </si>
   <si>
-    <t>alt_KOLF_PTO_GATCAGCTTACA_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_GATCAGCTTACA_r2.fq.gz</t>
-  </si>
-  <si>
     <t>alt_KOLF_PTO_GCTCAGAGACTT_r1.fq.gz</t>
   </si>
   <si>
     <t>alt_KOLF_PTO_GCTCAGAGACTT_r2.fq.gz</t>
   </si>
   <si>
-    <t>alt_KOLF_PTO_GGATTCACCGAA_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_GGATTCACCGAA_r2.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_GGCATTGTTCTG_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_GGCATTGTTCTG_r2.fq.gz</t>
-  </si>
-  <si>
     <t>alt_KOLF_PTO_GGTGACAACGCA_r1.fq.gz</t>
   </si>
   <si>
@@ -3562,24 +3533,6 @@
     <t>alt_KOLF_PTO_TACAAGGCACAA_r2.fq.gz</t>
   </si>
   <si>
-    <t>alt_KOLF_PTO_TCTTATCCTCGA_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_TCTTATCCTCGA_r2.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_TGACACTCACCA_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_TGACACTCACCA_r2.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_TGTGCCAAGGTG_r1.fq.gz</t>
-  </si>
-  <si>
-    <t>alt_KOLF_PTO_TGTGCCAAGGTG_r2.fq.gz</t>
-  </si>
-  <si>
     <t>alt_KOLF_PTO_TTCTGTTGCGAA_r1.fq.gz</t>
   </si>
   <si>
@@ -3968,6 +3921,54 @@
   </si>
   <si>
     <t>poolsize2_920_4_4_TGTAGCTCGCTA_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_AACAGCGCCATG_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_AACAGCGCCATG_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_AGTAGTTAGCCG_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_AGTAGTTAGCCG_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_GATCAGCTTACA_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_GATCAGCTTACA_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_GGATTCACCGAA_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_GGATTCACCGAA_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_GGCATTGTTCTG_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_GGCATTGTTCTG_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_TCTTATCCTCGA_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_TCTTATCCTCGA_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_TGACACTCACCA_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_TGACACTCACCA_r2.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_TGTGCCAAGGTG_r1.fq.gz</t>
+  </si>
+  <si>
+    <t>alt_Liver_PTO_TGTGCCAAGGTG_r2.fq.gz</t>
   </si>
 </sst>
 </file>
@@ -16208,7 +16209,7 @@
         <v>115120</v>
       </c>
       <c r="C1082" t="str">
-        <f>LEFT(A1082, LEN(A1082)-22)</f>
+        <f t="shared" ref="C1082:C1145" si="0">LEFT(A1082, LEN(A1082)-22)</f>
         <v>alt_KOLF_old</v>
       </c>
     </row>
@@ -16220,7 +16221,7 @@
         <v>115120</v>
       </c>
       <c r="C1083" t="str">
-        <f t="shared" ref="C1083:C1146" si="0">LEFT(A1083, LEN(A1083)-22)</f>
+        <f t="shared" si="0"/>
         <v>alt_KOLF_old</v>
       </c>
     </row>
@@ -16397,7 +16398,7 @@
         <v>1156</v>
       </c>
       <c r="B1098">
-        <v>196087</v>
+        <v>279092</v>
       </c>
       <c r="C1098" t="str">
         <f t="shared" si="0"/>
@@ -16409,7 +16410,7 @@
         <v>1157</v>
       </c>
       <c r="B1099">
-        <v>196087</v>
+        <v>279092</v>
       </c>
       <c r="C1099" t="str">
         <f t="shared" si="0"/>
@@ -16421,7 +16422,7 @@
         <v>1158</v>
       </c>
       <c r="B1100">
-        <v>279092</v>
+        <v>243356</v>
       </c>
       <c r="C1100" t="str">
         <f t="shared" si="0"/>
@@ -16433,7 +16434,7 @@
         <v>1159</v>
       </c>
       <c r="B1101">
-        <v>279092</v>
+        <v>243356</v>
       </c>
       <c r="C1101" t="str">
         <f t="shared" si="0"/>
@@ -16445,7 +16446,7 @@
         <v>1160</v>
       </c>
       <c r="B1102">
-        <v>243356</v>
+        <v>266064</v>
       </c>
       <c r="C1102" t="str">
         <f t="shared" si="0"/>
@@ -16457,7 +16458,7 @@
         <v>1161</v>
       </c>
       <c r="B1103">
-        <v>243356</v>
+        <v>266064</v>
       </c>
       <c r="C1103" t="str">
         <f t="shared" si="0"/>
@@ -16469,7 +16470,7 @@
         <v>1162</v>
       </c>
       <c r="B1104">
-        <v>193936</v>
+        <v>234687</v>
       </c>
       <c r="C1104" t="str">
         <f t="shared" si="0"/>
@@ -16481,7 +16482,7 @@
         <v>1163</v>
       </c>
       <c r="B1105">
-        <v>193936</v>
+        <v>234687</v>
       </c>
       <c r="C1105" t="str">
         <f t="shared" si="0"/>
@@ -16493,7 +16494,7 @@
         <v>1164</v>
       </c>
       <c r="B1106">
-        <v>266064</v>
+        <v>223970</v>
       </c>
       <c r="C1106" t="str">
         <f t="shared" si="0"/>
@@ -16505,7 +16506,7 @@
         <v>1165</v>
       </c>
       <c r="B1107">
-        <v>266064</v>
+        <v>223970</v>
       </c>
       <c r="C1107" t="str">
         <f t="shared" si="0"/>
@@ -16517,7 +16518,7 @@
         <v>1166</v>
       </c>
       <c r="B1108">
-        <v>234687</v>
+        <v>282370</v>
       </c>
       <c r="C1108" t="str">
         <f t="shared" si="0"/>
@@ -16529,7 +16530,7 @@
         <v>1167</v>
       </c>
       <c r="B1109">
-        <v>234687</v>
+        <v>282370</v>
       </c>
       <c r="C1109" t="str">
         <f t="shared" si="0"/>
@@ -16541,7 +16542,7 @@
         <v>1168</v>
       </c>
       <c r="B1110">
-        <v>318624</v>
+        <v>277899</v>
       </c>
       <c r="C1110" t="str">
         <f t="shared" si="0"/>
@@ -16553,7 +16554,7 @@
         <v>1169</v>
       </c>
       <c r="B1111">
-        <v>318624</v>
+        <v>277899</v>
       </c>
       <c r="C1111" t="str">
         <f t="shared" si="0"/>
@@ -16565,7 +16566,7 @@
         <v>1170</v>
       </c>
       <c r="B1112">
-        <v>223970</v>
+        <v>255616</v>
       </c>
       <c r="C1112" t="str">
         <f t="shared" si="0"/>
@@ -16577,7 +16578,7 @@
         <v>1171</v>
       </c>
       <c r="B1113">
-        <v>223970</v>
+        <v>255616</v>
       </c>
       <c r="C1113" t="str">
         <f t="shared" si="0"/>
@@ -16589,11 +16590,11 @@
         <v>1172</v>
       </c>
       <c r="B1114">
-        <v>292856</v>
+        <v>101311</v>
       </c>
       <c r="C1114" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1115" spans="1:3" x14ac:dyDescent="0.25">
@@ -16601,11 +16602,11 @@
         <v>1173</v>
       </c>
       <c r="B1115">
-        <v>292856</v>
+        <v>101311</v>
       </c>
       <c r="C1115" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1116" spans="1:3" x14ac:dyDescent="0.25">
@@ -16613,11 +16614,11 @@
         <v>1174</v>
       </c>
       <c r="B1116">
-        <v>119075</v>
+        <v>125737</v>
       </c>
       <c r="C1116" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1117" spans="1:3" x14ac:dyDescent="0.25">
@@ -16625,11 +16626,11 @@
         <v>1175</v>
       </c>
       <c r="B1117">
-        <v>119075</v>
+        <v>125737</v>
       </c>
       <c r="C1117" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1118" spans="1:3" x14ac:dyDescent="0.25">
@@ -16637,11 +16638,11 @@
         <v>1176</v>
       </c>
       <c r="B1118">
-        <v>282370</v>
+        <v>154553</v>
       </c>
       <c r="C1118" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1119" spans="1:3" x14ac:dyDescent="0.25">
@@ -16649,11 +16650,11 @@
         <v>1177</v>
       </c>
       <c r="B1119">
-        <v>282370</v>
+        <v>154553</v>
       </c>
       <c r="C1119" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1120" spans="1:3" x14ac:dyDescent="0.25">
@@ -16661,11 +16662,11 @@
         <v>1178</v>
       </c>
       <c r="B1120">
-        <v>277899</v>
+        <v>137875</v>
       </c>
       <c r="C1120" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1121" spans="1:3" x14ac:dyDescent="0.25">
@@ -16673,11 +16674,11 @@
         <v>1179</v>
       </c>
       <c r="B1121">
-        <v>277899</v>
+        <v>137875</v>
       </c>
       <c r="C1121" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1122" spans="1:3" x14ac:dyDescent="0.25">
@@ -16685,11 +16686,11 @@
         <v>1180</v>
       </c>
       <c r="B1122">
-        <v>319172</v>
+        <v>169525</v>
       </c>
       <c r="C1122" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1123" spans="1:3" x14ac:dyDescent="0.25">
@@ -16697,11 +16698,11 @@
         <v>1181</v>
       </c>
       <c r="B1123">
-        <v>319172</v>
+        <v>169525</v>
       </c>
       <c r="C1123" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1124" spans="1:3" x14ac:dyDescent="0.25">
@@ -16709,11 +16710,11 @@
         <v>1182</v>
       </c>
       <c r="B1124">
-        <v>255181</v>
+        <v>100222</v>
       </c>
       <c r="C1124" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1125" spans="1:3" x14ac:dyDescent="0.25">
@@ -16721,11 +16722,11 @@
         <v>1183</v>
       </c>
       <c r="B1125">
-        <v>255181</v>
+        <v>100222</v>
       </c>
       <c r="C1125" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1126" spans="1:3" x14ac:dyDescent="0.25">
@@ -16733,11 +16734,11 @@
         <v>1184</v>
       </c>
       <c r="B1126">
-        <v>128521</v>
+        <v>140528</v>
       </c>
       <c r="C1126" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1127" spans="1:3" x14ac:dyDescent="0.25">
@@ -16745,11 +16746,11 @@
         <v>1185</v>
       </c>
       <c r="B1127">
-        <v>128521</v>
+        <v>140528</v>
       </c>
       <c r="C1127" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1128" spans="1:3" x14ac:dyDescent="0.25">
@@ -16757,11 +16758,11 @@
         <v>1186</v>
       </c>
       <c r="B1128">
-        <v>255616</v>
+        <v>150490</v>
       </c>
       <c r="C1128" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1129" spans="1:3" x14ac:dyDescent="0.25">
@@ -16769,232 +16770,232 @@
         <v>1187</v>
       </c>
       <c r="B1129">
-        <v>255616</v>
+        <v>150490</v>
       </c>
       <c r="C1129" t="str">
         <f t="shared" si="0"/>
-        <v>alt_KOLF_PTO</v>
+        <v>alt_Liver_old</v>
       </c>
     </row>
     <row r="1130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1130" t="s">
-        <v>1188</v>
+        <v>1300</v>
       </c>
       <c r="B1130">
-        <v>101311</v>
+        <v>196087</v>
       </c>
       <c r="C1130" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1131" t="s">
-        <v>1189</v>
+        <v>1301</v>
       </c>
       <c r="B1131">
-        <v>101311</v>
+        <v>196087</v>
       </c>
       <c r="C1131" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1132" t="s">
-        <v>1190</v>
+        <v>1302</v>
       </c>
       <c r="B1132">
-        <v>125737</v>
+        <v>193936</v>
       </c>
       <c r="C1132" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1133" t="s">
-        <v>1191</v>
+        <v>1303</v>
       </c>
       <c r="B1133">
-        <v>125737</v>
+        <v>193936</v>
       </c>
       <c r="C1133" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1134" t="s">
-        <v>1192</v>
+        <v>1304</v>
       </c>
       <c r="B1134">
-        <v>154553</v>
+        <v>318624</v>
       </c>
       <c r="C1134" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1135" t="s">
-        <v>1193</v>
+        <v>1305</v>
       </c>
       <c r="B1135">
-        <v>154553</v>
+        <v>318624</v>
       </c>
       <c r="C1135" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1136" t="s">
-        <v>1194</v>
+        <v>1306</v>
       </c>
       <c r="B1136">
-        <v>137875</v>
+        <v>292856</v>
       </c>
       <c r="C1136" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1137" t="s">
-        <v>1195</v>
+        <v>1307</v>
       </c>
       <c r="B1137">
-        <v>137875</v>
+        <v>292856</v>
       </c>
       <c r="C1137" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1138" t="s">
-        <v>1196</v>
+        <v>1308</v>
       </c>
       <c r="B1138">
-        <v>169525</v>
+        <v>119075</v>
       </c>
       <c r="C1138" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1139" t="s">
-        <v>1197</v>
+        <v>1309</v>
       </c>
       <c r="B1139">
-        <v>169525</v>
+        <v>119075</v>
       </c>
       <c r="C1139" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1140" t="s">
-        <v>1198</v>
+        <v>1310</v>
       </c>
       <c r="B1140">
-        <v>100222</v>
+        <v>319172</v>
       </c>
       <c r="C1140" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1141" t="s">
-        <v>1199</v>
+        <v>1311</v>
       </c>
       <c r="B1141">
-        <v>100222</v>
+        <v>319172</v>
       </c>
       <c r="C1141" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1142" t="s">
-        <v>1200</v>
+        <v>1312</v>
       </c>
       <c r="B1142">
-        <v>140528</v>
+        <v>255181</v>
       </c>
       <c r="C1142" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1143" t="s">
-        <v>1201</v>
+        <v>1313</v>
       </c>
       <c r="B1143">
-        <v>140528</v>
+        <v>255181</v>
       </c>
       <c r="C1143" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1144" t="s">
-        <v>1202</v>
+        <v>1314</v>
       </c>
       <c r="B1144">
-        <v>150490</v>
+        <v>128521</v>
       </c>
       <c r="C1144" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1145" t="s">
-        <v>1203</v>
+        <v>1315</v>
       </c>
       <c r="B1145">
-        <v>150490</v>
+        <v>128521</v>
       </c>
       <c r="C1145" t="str">
         <f t="shared" si="0"/>
-        <v>alt_Liver_old</v>
+        <v>alt_Liver_PTO</v>
       </c>
     </row>
     <row r="1146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1146" t="s">
-        <v>1204</v>
+        <v>1188</v>
       </c>
       <c r="B1146">
         <v>955673</v>
       </c>
       <c r="C1146" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C1146:C1209" si="1">LEFT(A1146, LEN(A1146)-22)</f>
         <v>poolsize2_80_1_1</v>
       </c>
     </row>
     <row r="1147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1147" t="s">
-        <v>1205</v>
+        <v>1189</v>
       </c>
       <c r="B1147">
         <v>955673</v>
       </c>
       <c r="C1147" t="str">
-        <f t="shared" ref="C1147:C1210" si="1">LEFT(A1147, LEN(A1147)-22)</f>
+        <f t="shared" si="1"/>
         <v>poolsize2_80_1_1</v>
       </c>
     </row>
     <row r="1148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1148" t="s">
-        <v>1206</v>
+        <v>1190</v>
       </c>
       <c r="B1148">
         <v>1208351</v>
@@ -17006,7 +17007,7 @@
     </row>
     <row r="1149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1149" t="s">
-        <v>1207</v>
+        <v>1191</v>
       </c>
       <c r="B1149">
         <v>1208351</v>
@@ -17018,7 +17019,7 @@
     </row>
     <row r="1150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1150" t="s">
-        <v>1208</v>
+        <v>1192</v>
       </c>
       <c r="B1150">
         <v>1311773</v>
@@ -17030,7 +17031,7 @@
     </row>
     <row r="1151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1151" t="s">
-        <v>1209</v>
+        <v>1193</v>
       </c>
       <c r="B1151">
         <v>1311773</v>
@@ -17042,7 +17043,7 @@
     </row>
     <row r="1152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1152" t="s">
-        <v>1210</v>
+        <v>1194</v>
       </c>
       <c r="B1152">
         <v>1124142</v>
@@ -17054,7 +17055,7 @@
     </row>
     <row r="1153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1153" t="s">
-        <v>1211</v>
+        <v>1195</v>
       </c>
       <c r="B1153">
         <v>1124142</v>
@@ -17066,7 +17067,7 @@
     </row>
     <row r="1154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1154" t="s">
-        <v>1212</v>
+        <v>1196</v>
       </c>
       <c r="B1154">
         <v>1053665</v>
@@ -17078,7 +17079,7 @@
     </row>
     <row r="1155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1155" t="s">
-        <v>1213</v>
+        <v>1197</v>
       </c>
       <c r="B1155">
         <v>1053665</v>
@@ -17090,7 +17091,7 @@
     </row>
     <row r="1156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1156" t="s">
-        <v>1214</v>
+        <v>1198</v>
       </c>
       <c r="B1156">
         <v>1145674</v>
@@ -17102,7 +17103,7 @@
     </row>
     <row r="1157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1157" t="s">
-        <v>1215</v>
+        <v>1199</v>
       </c>
       <c r="B1157">
         <v>1145674</v>
@@ -17114,7 +17115,7 @@
     </row>
     <row r="1158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1158" t="s">
-        <v>1216</v>
+        <v>1200</v>
       </c>
       <c r="B1158">
         <v>1112367</v>
@@ -17126,7 +17127,7 @@
     </row>
     <row r="1159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1159" t="s">
-        <v>1217</v>
+        <v>1201</v>
       </c>
       <c r="B1159">
         <v>1112367</v>
@@ -17138,7 +17139,7 @@
     </row>
     <row r="1160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1160" t="s">
-        <v>1218</v>
+        <v>1202</v>
       </c>
       <c r="B1160">
         <v>1013102</v>
@@ -17150,7 +17151,7 @@
     </row>
     <row r="1161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1161" t="s">
-        <v>1219</v>
+        <v>1203</v>
       </c>
       <c r="B1161">
         <v>1013102</v>
@@ -17162,7 +17163,7 @@
     </row>
     <row r="1162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1162" t="s">
-        <v>1220</v>
+        <v>1204</v>
       </c>
       <c r="B1162">
         <v>1042385</v>
@@ -17174,7 +17175,7 @@
     </row>
     <row r="1163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1163" t="s">
-        <v>1221</v>
+        <v>1205</v>
       </c>
       <c r="B1163">
         <v>1042385</v>
@@ -17186,7 +17187,7 @@
     </row>
     <row r="1164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1164" t="s">
-        <v>1222</v>
+        <v>1206</v>
       </c>
       <c r="B1164">
         <v>1312505</v>
@@ -17198,7 +17199,7 @@
     </row>
     <row r="1165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1165" t="s">
-        <v>1223</v>
+        <v>1207</v>
       </c>
       <c r="B1165">
         <v>1312505</v>
@@ -17210,7 +17211,7 @@
     </row>
     <row r="1166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1166" t="s">
-        <v>1224</v>
+        <v>1208</v>
       </c>
       <c r="B1166">
         <v>1224014</v>
@@ -17222,7 +17223,7 @@
     </row>
     <row r="1167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1167" t="s">
-        <v>1225</v>
+        <v>1209</v>
       </c>
       <c r="B1167">
         <v>1224014</v>
@@ -17234,7 +17235,7 @@
     </row>
     <row r="1168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1168" t="s">
-        <v>1226</v>
+        <v>1210</v>
       </c>
       <c r="B1168">
         <v>1159244</v>
@@ -17246,7 +17247,7 @@
     </row>
     <row r="1169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1169" t="s">
-        <v>1227</v>
+        <v>1211</v>
       </c>
       <c r="B1169">
         <v>1159244</v>
@@ -17258,7 +17259,7 @@
     </row>
     <row r="1170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1170" t="s">
-        <v>1228</v>
+        <v>1212</v>
       </c>
       <c r="B1170">
         <v>1422335</v>
@@ -17270,7 +17271,7 @@
     </row>
     <row r="1171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1171" t="s">
-        <v>1229</v>
+        <v>1213</v>
       </c>
       <c r="B1171">
         <v>1422335</v>
@@ -17282,7 +17283,7 @@
     </row>
     <row r="1172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1172" t="s">
-        <v>1230</v>
+        <v>1214</v>
       </c>
       <c r="B1172">
         <v>1001108</v>
@@ -17294,7 +17295,7 @@
     </row>
     <row r="1173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1173" t="s">
-        <v>1231</v>
+        <v>1215</v>
       </c>
       <c r="B1173">
         <v>1001108</v>
@@ -17306,7 +17307,7 @@
     </row>
     <row r="1174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1174" t="s">
-        <v>1232</v>
+        <v>1216</v>
       </c>
       <c r="B1174">
         <v>1356215</v>
@@ -17318,7 +17319,7 @@
     </row>
     <row r="1175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1175" t="s">
-        <v>1233</v>
+        <v>1217</v>
       </c>
       <c r="B1175">
         <v>1356215</v>
@@ -17330,7 +17331,7 @@
     </row>
     <row r="1176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1176" t="s">
-        <v>1234</v>
+        <v>1218</v>
       </c>
       <c r="B1176">
         <v>1293182</v>
@@ -17342,7 +17343,7 @@
     </row>
     <row r="1177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1177" t="s">
-        <v>1235</v>
+        <v>1219</v>
       </c>
       <c r="B1177">
         <v>1293182</v>
@@ -17354,7 +17355,7 @@
     </row>
     <row r="1178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1178" t="s">
-        <v>1236</v>
+        <v>1220</v>
       </c>
       <c r="B1178">
         <v>957167</v>
@@ -17366,7 +17367,7 @@
     </row>
     <row r="1179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1179" t="s">
-        <v>1237</v>
+        <v>1221</v>
       </c>
       <c r="B1179">
         <v>957167</v>
@@ -17378,7 +17379,7 @@
     </row>
     <row r="1180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1180" t="s">
-        <v>1238</v>
+        <v>1222</v>
       </c>
       <c r="B1180">
         <v>1317532</v>
@@ -17390,7 +17391,7 @@
     </row>
     <row r="1181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1181" t="s">
-        <v>1239</v>
+        <v>1223</v>
       </c>
       <c r="B1181">
         <v>1317532</v>
@@ -17402,7 +17403,7 @@
     </row>
     <row r="1182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1182" t="s">
-        <v>1240</v>
+        <v>1224</v>
       </c>
       <c r="B1182">
         <v>1294685</v>
@@ -17414,7 +17415,7 @@
     </row>
     <row r="1183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1183" t="s">
-        <v>1241</v>
+        <v>1225</v>
       </c>
       <c r="B1183">
         <v>1294685</v>
@@ -17426,7 +17427,7 @@
     </row>
     <row r="1184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1184" t="s">
-        <v>1242</v>
+        <v>1226</v>
       </c>
       <c r="B1184">
         <v>1418706</v>
@@ -17438,7 +17439,7 @@
     </row>
     <row r="1185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1185" t="s">
-        <v>1243</v>
+        <v>1227</v>
       </c>
       <c r="B1185">
         <v>1418706</v>
@@ -17450,7 +17451,7 @@
     </row>
     <row r="1186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1186" t="s">
-        <v>1244</v>
+        <v>1228</v>
       </c>
       <c r="B1186">
         <v>1077472</v>
@@ -17462,7 +17463,7 @@
     </row>
     <row r="1187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1187" t="s">
-        <v>1245</v>
+        <v>1229</v>
       </c>
       <c r="B1187">
         <v>1077472</v>
@@ -17474,7 +17475,7 @@
     </row>
     <row r="1188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1188" t="s">
-        <v>1246</v>
+        <v>1230</v>
       </c>
       <c r="B1188">
         <v>1216453</v>
@@ -17486,7 +17487,7 @@
     </row>
     <row r="1189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1189" t="s">
-        <v>1247</v>
+        <v>1231</v>
       </c>
       <c r="B1189">
         <v>1216453</v>
@@ -17498,7 +17499,7 @@
     </row>
     <row r="1190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1190" t="s">
-        <v>1248</v>
+        <v>1232</v>
       </c>
       <c r="B1190">
         <v>1258902</v>
@@ -17510,7 +17511,7 @@
     </row>
     <row r="1191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1191" t="s">
-        <v>1249</v>
+        <v>1233</v>
       </c>
       <c r="B1191">
         <v>1258902</v>
@@ -17522,7 +17523,7 @@
     </row>
     <row r="1192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1192" t="s">
-        <v>1250</v>
+        <v>1234</v>
       </c>
       <c r="B1192">
         <v>1284399</v>
@@ -17534,7 +17535,7 @@
     </row>
     <row r="1193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1193" t="s">
-        <v>1251</v>
+        <v>1235</v>
       </c>
       <c r="B1193">
         <v>1284399</v>
@@ -17546,7 +17547,7 @@
     </row>
     <row r="1194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1194" t="s">
-        <v>1252</v>
+        <v>1236</v>
       </c>
       <c r="B1194">
         <v>1080846</v>
@@ -17558,7 +17559,7 @@
     </row>
     <row r="1195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1195" t="s">
-        <v>1253</v>
+        <v>1237</v>
       </c>
       <c r="B1195">
         <v>1080846</v>
@@ -17570,7 +17571,7 @@
     </row>
     <row r="1196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1196" t="s">
-        <v>1254</v>
+        <v>1238</v>
       </c>
       <c r="B1196">
         <v>1205068</v>
@@ -17582,7 +17583,7 @@
     </row>
     <row r="1197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1197" t="s">
-        <v>1255</v>
+        <v>1239</v>
       </c>
       <c r="B1197">
         <v>1205068</v>
@@ -17594,7 +17595,7 @@
     </row>
     <row r="1198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1198" t="s">
-        <v>1256</v>
+        <v>1240</v>
       </c>
       <c r="B1198">
         <v>1188511</v>
@@ -17606,7 +17607,7 @@
     </row>
     <row r="1199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1199" t="s">
-        <v>1257</v>
+        <v>1241</v>
       </c>
       <c r="B1199">
         <v>1188511</v>
@@ -17618,7 +17619,7 @@
     </row>
     <row r="1200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1200" t="s">
-        <v>1258</v>
+        <v>1242</v>
       </c>
       <c r="B1200">
         <v>1243920</v>
@@ -17630,7 +17631,7 @@
     </row>
     <row r="1201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1201" t="s">
-        <v>1259</v>
+        <v>1243</v>
       </c>
       <c r="B1201">
         <v>1243920</v>
@@ -17642,7 +17643,7 @@
     </row>
     <row r="1202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1202" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
       <c r="B1202">
         <v>1273648</v>
@@ -17654,7 +17655,7 @@
     </row>
     <row r="1203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1203" t="s">
-        <v>1261</v>
+        <v>1245</v>
       </c>
       <c r="B1203">
         <v>1273648</v>
@@ -17666,7 +17667,7 @@
     </row>
     <row r="1204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1204" t="s">
-        <v>1262</v>
+        <v>1246</v>
       </c>
       <c r="B1204">
         <v>1028181</v>
@@ -17678,7 +17679,7 @@
     </row>
     <row r="1205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1205" t="s">
-        <v>1263</v>
+        <v>1247</v>
       </c>
       <c r="B1205">
         <v>1028181</v>
@@ -17690,7 +17691,7 @@
     </row>
     <row r="1206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1206" t="s">
-        <v>1264</v>
+        <v>1248</v>
       </c>
       <c r="B1206">
         <v>1283042</v>
@@ -17702,7 +17703,7 @@
     </row>
     <row r="1207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1207" t="s">
-        <v>1265</v>
+        <v>1249</v>
       </c>
       <c r="B1207">
         <v>1283042</v>
@@ -17714,7 +17715,7 @@
     </row>
     <row r="1208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1208" t="s">
-        <v>1266</v>
+        <v>1250</v>
       </c>
       <c r="B1208">
         <v>1207413</v>
@@ -17726,7 +17727,7 @@
     </row>
     <row r="1209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1209" t="s">
-        <v>1267</v>
+        <v>1251</v>
       </c>
       <c r="B1209">
         <v>1207413</v>
@@ -17738,31 +17739,31 @@
     </row>
     <row r="1210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1210" t="s">
-        <v>1268</v>
+        <v>1252</v>
       </c>
       <c r="B1210">
         <v>1017381</v>
       </c>
       <c r="C1210" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="C1210:C1257" si="2">LEFT(A1210, LEN(A1210)-22)</f>
         <v>poolsize2_920_1_4</v>
       </c>
     </row>
     <row r="1211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1211" t="s">
-        <v>1269</v>
+        <v>1253</v>
       </c>
       <c r="B1211">
         <v>1017381</v>
       </c>
       <c r="C1211" t="str">
-        <f t="shared" ref="C1211:C1257" si="2">LEFT(A1211, LEN(A1211)-22)</f>
+        <f t="shared" si="2"/>
         <v>poolsize2_920_1_4</v>
       </c>
     </row>
     <row r="1212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1212" t="s">
-        <v>1270</v>
+        <v>1254</v>
       </c>
       <c r="B1212">
         <v>1222173</v>
@@ -17774,7 +17775,7 @@
     </row>
     <row r="1213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1213" t="s">
-        <v>1271</v>
+        <v>1255</v>
       </c>
       <c r="B1213">
         <v>1222173</v>
@@ -17786,7 +17787,7 @@
     </row>
     <row r="1214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1214" t="s">
-        <v>1272</v>
+        <v>1256</v>
       </c>
       <c r="B1214">
         <v>1228167</v>
@@ -17798,7 +17799,7 @@
     </row>
     <row r="1215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1215" t="s">
-        <v>1273</v>
+        <v>1257</v>
       </c>
       <c r="B1215">
         <v>1228167</v>
@@ -17810,7 +17811,7 @@
     </row>
     <row r="1216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1216" t="s">
-        <v>1274</v>
+        <v>1258</v>
       </c>
       <c r="B1216">
         <v>1332371</v>
@@ -17822,7 +17823,7 @@
     </row>
     <row r="1217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1217" t="s">
-        <v>1275</v>
+        <v>1259</v>
       </c>
       <c r="B1217">
         <v>1332371</v>
@@ -17834,7 +17835,7 @@
     </row>
     <row r="1218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1218" t="s">
-        <v>1276</v>
+        <v>1260</v>
       </c>
       <c r="B1218">
         <v>1015366</v>
@@ -17846,7 +17847,7 @@
     </row>
     <row r="1219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1219" t="s">
-        <v>1277</v>
+        <v>1261</v>
       </c>
       <c r="B1219">
         <v>1015366</v>
@@ -17858,7 +17859,7 @@
     </row>
     <row r="1220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1220" t="s">
-        <v>1278</v>
+        <v>1262</v>
       </c>
       <c r="B1220">
         <v>1180018</v>
@@ -17870,7 +17871,7 @@
     </row>
     <row r="1221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1221" t="s">
-        <v>1279</v>
+        <v>1263</v>
       </c>
       <c r="B1221">
         <v>1180018</v>
@@ -17882,7 +17883,7 @@
     </row>
     <row r="1222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1222" t="s">
-        <v>1280</v>
+        <v>1264</v>
       </c>
       <c r="B1222">
         <v>1178420</v>
@@ -17894,7 +17895,7 @@
     </row>
     <row r="1223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1223" t="s">
-        <v>1281</v>
+        <v>1265</v>
       </c>
       <c r="B1223">
         <v>1178420</v>
@@ -17906,7 +17907,7 @@
     </row>
     <row r="1224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1224" t="s">
-        <v>1282</v>
+        <v>1266</v>
       </c>
       <c r="B1224">
         <v>1203835</v>
@@ -17918,7 +17919,7 @@
     </row>
     <row r="1225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1225" t="s">
-        <v>1283</v>
+        <v>1267</v>
       </c>
       <c r="B1225">
         <v>1203835</v>
@@ -17930,7 +17931,7 @@
     </row>
     <row r="1226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1226" t="s">
-        <v>1284</v>
+        <v>1268</v>
       </c>
       <c r="B1226">
         <v>1018446</v>
@@ -17942,7 +17943,7 @@
     </row>
     <row r="1227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1227" t="s">
-        <v>1285</v>
+        <v>1269</v>
       </c>
       <c r="B1227">
         <v>1018446</v>
@@ -17954,7 +17955,7 @@
     </row>
     <row r="1228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1228" t="s">
-        <v>1286</v>
+        <v>1270</v>
       </c>
       <c r="B1228">
         <v>1228094</v>
@@ -17966,7 +17967,7 @@
     </row>
     <row r="1229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1229" t="s">
-        <v>1287</v>
+        <v>1271</v>
       </c>
       <c r="B1229">
         <v>1228094</v>
@@ -17978,7 +17979,7 @@
     </row>
     <row r="1230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1230" t="s">
-        <v>1288</v>
+        <v>1272</v>
       </c>
       <c r="B1230">
         <v>1135968</v>
@@ -17990,7 +17991,7 @@
     </row>
     <row r="1231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1231" t="s">
-        <v>1289</v>
+        <v>1273</v>
       </c>
       <c r="B1231">
         <v>1135968</v>
@@ -18002,7 +18003,7 @@
     </row>
     <row r="1232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1232" t="s">
-        <v>1290</v>
+        <v>1274</v>
       </c>
       <c r="B1232">
         <v>1236744</v>
@@ -18014,7 +18015,7 @@
     </row>
     <row r="1233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1233" t="s">
-        <v>1291</v>
+        <v>1275</v>
       </c>
       <c r="B1233">
         <v>1236744</v>
@@ -18026,7 +18027,7 @@
     </row>
     <row r="1234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1234" t="s">
-        <v>1292</v>
+        <v>1276</v>
       </c>
       <c r="B1234">
         <v>967673</v>
@@ -18038,7 +18039,7 @@
     </row>
     <row r="1235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1235" t="s">
-        <v>1293</v>
+        <v>1277</v>
       </c>
       <c r="B1235">
         <v>967673</v>
@@ -18050,7 +18051,7 @@
     </row>
     <row r="1236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1236" t="s">
-        <v>1294</v>
+        <v>1278</v>
       </c>
       <c r="B1236">
         <v>888749</v>
@@ -18062,7 +18063,7 @@
     </row>
     <row r="1237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1237" t="s">
-        <v>1295</v>
+        <v>1279</v>
       </c>
       <c r="B1237">
         <v>888749</v>
@@ -18074,7 +18075,7 @@
     </row>
     <row r="1238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1238" t="s">
-        <v>1296</v>
+        <v>1280</v>
       </c>
       <c r="B1238">
         <v>1232188</v>
@@ -18086,7 +18087,7 @@
     </row>
     <row r="1239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1239" t="s">
-        <v>1297</v>
+        <v>1281</v>
       </c>
       <c r="B1239">
         <v>1232188</v>
@@ -18098,7 +18099,7 @@
     </row>
     <row r="1240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1240" t="s">
-        <v>1298</v>
+        <v>1282</v>
       </c>
       <c r="B1240">
         <v>1166769</v>
@@ -18110,7 +18111,7 @@
     </row>
     <row r="1241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1241" t="s">
-        <v>1299</v>
+        <v>1283</v>
       </c>
       <c r="B1241">
         <v>1166769</v>
@@ -18122,7 +18123,7 @@
     </row>
     <row r="1242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1242" t="s">
-        <v>1300</v>
+        <v>1284</v>
       </c>
       <c r="B1242">
         <v>950689</v>
@@ -18134,7 +18135,7 @@
     </row>
     <row r="1243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1243" t="s">
-        <v>1301</v>
+        <v>1285</v>
       </c>
       <c r="B1243">
         <v>950689</v>
@@ -18146,7 +18147,7 @@
     </row>
     <row r="1244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1244" t="s">
-        <v>1302</v>
+        <v>1286</v>
       </c>
       <c r="B1244">
         <v>1134572</v>
@@ -18158,7 +18159,7 @@
     </row>
     <row r="1245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1245" t="s">
-        <v>1303</v>
+        <v>1287</v>
       </c>
       <c r="B1245">
         <v>1134572</v>
@@ -18170,7 +18171,7 @@
     </row>
     <row r="1246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1246" t="s">
-        <v>1304</v>
+        <v>1288</v>
       </c>
       <c r="B1246">
         <v>1173596</v>
@@ -18182,7 +18183,7 @@
     </row>
     <row r="1247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1247" t="s">
-        <v>1305</v>
+        <v>1289</v>
       </c>
       <c r="B1247">
         <v>1173596</v>
@@ -18194,7 +18195,7 @@
     </row>
     <row r="1248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1248" t="s">
-        <v>1306</v>
+        <v>1290</v>
       </c>
       <c r="B1248">
         <v>1365096</v>
@@ -18206,7 +18207,7 @@
     </row>
     <row r="1249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1249" t="s">
-        <v>1307</v>
+        <v>1291</v>
       </c>
       <c r="B1249">
         <v>1365096</v>
@@ -18218,7 +18219,7 @@
     </row>
     <row r="1250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1250" t="s">
-        <v>1308</v>
+        <v>1292</v>
       </c>
       <c r="B1250">
         <v>1038917</v>
@@ -18230,7 +18231,7 @@
     </row>
     <row r="1251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1251" t="s">
-        <v>1309</v>
+        <v>1293</v>
       </c>
       <c r="B1251">
         <v>1038917</v>
@@ -18242,7 +18243,7 @@
     </row>
     <row r="1252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1252" t="s">
-        <v>1310</v>
+        <v>1294</v>
       </c>
       <c r="B1252">
         <v>1093903</v>
@@ -18254,7 +18255,7 @@
     </row>
     <row r="1253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1253" t="s">
-        <v>1311</v>
+        <v>1295</v>
       </c>
       <c r="B1253">
         <v>1093903</v>
@@ -18266,7 +18267,7 @@
     </row>
     <row r="1254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1254" t="s">
-        <v>1312</v>
+        <v>1296</v>
       </c>
       <c r="B1254">
         <v>1176975</v>
@@ -18278,7 +18279,7 @@
     </row>
     <row r="1255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1255" t="s">
-        <v>1313</v>
+        <v>1297</v>
       </c>
       <c r="B1255">
         <v>1176975</v>
@@ -18290,7 +18291,7 @@
     </row>
     <row r="1256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1256" t="s">
-        <v>1314</v>
+        <v>1298</v>
       </c>
       <c r="B1256">
         <v>1148530</v>
@@ -18302,7 +18303,7 @@
     </row>
     <row r="1257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1257" t="s">
-        <v>1315</v>
+        <v>1299</v>
       </c>
       <c r="B1257">
         <v>1148530</v>

</xml_diff>